<commit_message>
very very messy code, just trying things out for now
</commit_message>
<xml_diff>
--- a/spreadsheets/P_lanceolata.xlsx
+++ b/spreadsheets/P_lanceolata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sallyborrowman/R_projects/temporal_pollinators/spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB0A2EA-B2F9-7A41-989F-197D8CDE7F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFA9DD3-8705-A844-8604-45DA1F4936BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{DD5157BD-592B-EF4A-95FF-FB179A475922}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="17400" activeTab="1" xr2:uid="{DD5157BD-592B-EF4A-95FF-FB179A475922}"/>
   </bookViews>
   <sheets>
     <sheet name="pollinator_data_raw" sheetId="1" r:id="rId1"/>
@@ -118,15 +118,6 @@
     <t xml:space="preserve">number_of_plantago </t>
   </si>
   <si>
-    <t xml:space="preserve">pollinators/flower </t>
-  </si>
-  <si>
-    <t>pollinators/flower/minute</t>
-  </si>
-  <si>
-    <t>plantago/m2</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
@@ -200,6 +191,15 @@
   </si>
   <si>
     <t xml:space="preserve">Apis_meliffera </t>
+  </si>
+  <si>
+    <t xml:space="preserve">pollinators_per_flower </t>
+  </si>
+  <si>
+    <t>pollinators_flower_minute</t>
+  </si>
+  <si>
+    <t>plantago_per_m2</t>
   </si>
 </sst>
 </file>
@@ -647,7 +647,7 @@
         <v>46196</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D2">
         <v>621.20000000000005</v>
@@ -688,7 +688,7 @@
         <v>46196</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D3">
         <v>621.20000000000005</v>
@@ -729,7 +729,7 @@
         <v>46196</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D4">
         <v>375</v>
@@ -756,7 +756,7 @@
         <v>0.75902777777777775</v>
       </c>
       <c r="M4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -767,7 +767,7 @@
         <v>46197</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D5">
         <v>586.25</v>
@@ -808,7 +808,7 @@
         <v>46197</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D6">
         <v>586.25</v>
@@ -835,7 +835,7 @@
         <v>0.42638888888888887</v>
       </c>
       <c r="M6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -846,7 +846,7 @@
         <v>46197</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D7">
         <v>883.25</v>
@@ -873,7 +873,7 @@
         <v>0.49722222222222223</v>
       </c>
       <c r="M7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -884,7 +884,7 @@
         <v>46202</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D8">
         <v>486.625</v>
@@ -922,7 +922,7 @@
         <v>46202</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D9">
         <v>486.625</v>
@@ -960,7 +960,7 @@
         <v>46202</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D10">
         <v>486.625</v>
@@ -987,7 +987,7 @@
         <v>0.36041666666666666</v>
       </c>
       <c r="M10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -998,7 +998,7 @@
         <v>46202</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D11">
         <v>486.625</v>
@@ -1025,7 +1025,7 @@
         <v>0.39374999999999999</v>
       </c>
       <c r="M11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -1036,7 +1036,7 @@
         <v>46202</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D12">
         <v>721.5</v>
@@ -1074,7 +1074,7 @@
         <v>46204</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D13">
         <v>154.17500000000001</v>
@@ -1112,7 +1112,7 @@
         <v>46204</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D14">
         <v>78.7</v>
@@ -1150,7 +1150,7 @@
         <v>46205</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D15">
         <v>562.25</v>
@@ -1188,7 +1188,7 @@
         <v>46205</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D16">
         <v>115.55</v>
@@ -1226,7 +1226,7 @@
         <v>46206</v>
       </c>
       <c r="C17" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D17">
         <v>405.75</v>
@@ -1264,7 +1264,7 @@
         <v>46206</v>
       </c>
       <c r="C18" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D18">
         <v>664</v>
@@ -1302,7 +1302,7 @@
         <v>46209</v>
       </c>
       <c r="C19" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D19">
         <v>69.224999999999994</v>
@@ -1329,7 +1329,7 @@
         <v>0.37152777777777779</v>
       </c>
       <c r="M19" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
@@ -1340,7 +1340,7 @@
         <v>46209</v>
       </c>
       <c r="C20" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D20">
         <v>69.224999999999994</v>
@@ -1367,7 +1367,7 @@
         <v>0.42986111111111114</v>
       </c>
       <c r="M20" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
@@ -1378,7 +1378,7 @@
         <v>46209</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D21">
         <v>95.924999999999983</v>
@@ -1416,7 +1416,7 @@
         <v>46210</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D22">
         <v>307.65000000000003</v>
@@ -1454,7 +1454,7 @@
         <v>46210</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D23">
         <v>93.325000000000003</v>
@@ -1481,7 +1481,7 @@
         <v>0.78819444444444442</v>
       </c>
       <c r="M23" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
@@ -1492,7 +1492,7 @@
         <v>46212</v>
       </c>
       <c r="C24" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D24">
         <v>690.75</v>
@@ -1519,7 +1519,7 @@
         <v>0.41180555555555554</v>
       </c>
       <c r="M24" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
@@ -1530,7 +1530,7 @@
         <v>46212</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D25">
         <v>806.75</v>
@@ -1557,7 +1557,7 @@
         <v>0.51736111111111116</v>
       </c>
       <c r="M25" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="N25" t="s">
         <v>17</v>
@@ -1571,7 +1571,7 @@
         <v>46213</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D26">
         <v>737.5</v>
@@ -1609,7 +1609,7 @@
         <v>46213</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D27">
         <v>422.25</v>
@@ -1636,7 +1636,7 @@
         <v>0.75972222222222219</v>
       </c>
       <c r="M27" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
@@ -1647,7 +1647,7 @@
         <v>46216</v>
       </c>
       <c r="C28" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D28">
         <v>461.375</v>
@@ -1685,7 +1685,7 @@
         <v>46216</v>
       </c>
       <c r="C29" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D29">
         <v>915</v>
@@ -1723,7 +1723,7 @@
         <v>46217</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D30">
         <v>641.5</v>
@@ -1750,7 +1750,7 @@
         <v>0.60833333333333328</v>
       </c>
       <c r="M30" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
@@ -1761,7 +1761,7 @@
         <v>46217</v>
       </c>
       <c r="C31" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D31">
         <v>641.5</v>
@@ -1788,7 +1788,7 @@
         <v>0.61527777777777781</v>
       </c>
       <c r="M31" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="N31" t="s">
         <v>16</v>
@@ -1802,7 +1802,7 @@
         <v>46217</v>
       </c>
       <c r="C32" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D32">
         <v>564.75</v>
@@ -1840,7 +1840,7 @@
         <v>46219</v>
       </c>
       <c r="C33" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D33">
         <v>220.42500000000001</v>
@@ -1867,7 +1867,7 @@
         <v>0.34513888888888888</v>
       </c>
       <c r="M33" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="N33" t="s">
         <v>16</v>
@@ -1881,7 +1881,7 @@
         <v>46219</v>
       </c>
       <c r="C34" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D34">
         <v>220.42500000000001</v>
@@ -1908,7 +1908,7 @@
         <v>0.3659722222222222</v>
       </c>
       <c r="M34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
@@ -1919,7 +1919,7 @@
         <v>46219</v>
       </c>
       <c r="C35" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D35">
         <v>220.42500000000001</v>
@@ -1946,7 +1946,7 @@
         <v>0.38055555555555554</v>
       </c>
       <c r="M35" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="N35" t="s">
         <v>16</v>
@@ -1960,7 +1960,7 @@
         <v>46219</v>
       </c>
       <c r="C36" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D36">
         <v>750</v>
@@ -1987,7 +1987,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="M36" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="N36" t="s">
         <v>17</v>
@@ -2001,7 +2001,7 @@
         <v>46251</v>
       </c>
       <c r="C37" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D37">
         <v>835.25</v>
@@ -2028,7 +2028,7 @@
         <v>0.64027777777777772</v>
       </c>
       <c r="M37" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="N37" t="s">
         <v>16</v>
@@ -2042,7 +2042,7 @@
         <v>46251</v>
       </c>
       <c r="C38" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D38">
         <v>548.5</v>
@@ -2133,13 +2133,13 @@
         <v>25</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -2150,7 +2150,7 @@
         <v>46196</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D2">
         <v>621.20000000000005</v>
@@ -2197,7 +2197,7 @@
         <v>46196</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D3">
         <v>375</v>
@@ -2244,7 +2244,7 @@
         <v>46197</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D4">
         <v>586.25</v>
@@ -2291,7 +2291,7 @@
         <v>46197</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D5">
         <v>883.25</v>
@@ -2338,7 +2338,7 @@
         <v>46202</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D6">
         <v>486.625</v>
@@ -2385,7 +2385,7 @@
         <v>46202</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D7">
         <v>721.5</v>
@@ -2432,7 +2432,7 @@
         <v>46204</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D8">
         <v>154.17500000000001</v>
@@ -2479,7 +2479,7 @@
         <v>46204</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D9">
         <v>78.7</v>
@@ -2526,7 +2526,7 @@
         <v>46205</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D10">
         <v>562.25</v>
@@ -2573,7 +2573,7 @@
         <v>46205</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D11">
         <v>115.55</v>
@@ -2620,7 +2620,7 @@
         <v>46206</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D12">
         <v>405.75</v>
@@ -2667,7 +2667,7 @@
         <v>46206</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D13">
         <v>664</v>
@@ -2714,7 +2714,7 @@
         <v>46209</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D14">
         <v>69.224999999999994</v>
@@ -2761,7 +2761,7 @@
         <v>46209</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D15">
         <v>95.924999999999983</v>
@@ -2808,7 +2808,7 @@
         <v>46210</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D16">
         <v>307.65000000000003</v>
@@ -2855,7 +2855,7 @@
         <v>46210</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D17">
         <v>93.325000000000003</v>
@@ -2902,7 +2902,7 @@
         <v>46212</v>
       </c>
       <c r="C18" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D18">
         <v>690.75</v>
@@ -2949,7 +2949,7 @@
         <v>46212</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D19">
         <v>806.75</v>
@@ -2996,7 +2996,7 @@
         <v>46213</v>
       </c>
       <c r="C20" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D20">
         <v>737.5</v>
@@ -3043,7 +3043,7 @@
         <v>46213</v>
       </c>
       <c r="C21" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D21">
         <v>422.25</v>
@@ -3090,7 +3090,7 @@
         <v>46216</v>
       </c>
       <c r="C22" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D22">
         <v>461.375</v>
@@ -3137,7 +3137,7 @@
         <v>46216</v>
       </c>
       <c r="C23" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D23">
         <v>915</v>
@@ -3184,7 +3184,7 @@
         <v>46217</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D24">
         <v>641.5</v>
@@ -3231,7 +3231,7 @@
         <v>46217</v>
       </c>
       <c r="C25" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D25">
         <v>564.75</v>
@@ -3278,7 +3278,7 @@
         <v>46219</v>
       </c>
       <c r="C26" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D26">
         <v>220.42500000000001</v>
@@ -3325,7 +3325,7 @@
         <v>46219</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D27">
         <v>750</v>
@@ -3372,7 +3372,7 @@
         <v>46251</v>
       </c>
       <c r="C28" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D28">
         <v>835.25</v>
@@ -3419,7 +3419,7 @@
         <v>46251</v>
       </c>
       <c r="C29" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D29">
         <v>548.5</v>
@@ -3486,34 +3486,34 @@
         <v>19</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
new r script thats better and changes in old one.
</commit_message>
<xml_diff>
--- a/spreadsheets/P_lanceolata.xlsx
+++ b/spreadsheets/P_lanceolata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sallyborrowman/R_projects/temporal_pollinators/spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFA9DD3-8705-A844-8604-45DA1F4936BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EE88B7-4708-4943-946F-9FC35F34C279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="17400" activeTab="1" xr2:uid="{DD5157BD-592B-EF4A-95FF-FB179A475922}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="number_of_pollinators" sheetId="2" r:id="rId2"/>
     <sheet name="floral_units" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -242,11 +242,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -589,6 +590,7 @@
     <col min="5" max="5" width="15.33203125" customWidth="1"/>
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="19.5" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" customWidth="1"/>
     <col min="11" max="11" width="23.83203125" customWidth="1"/>
     <col min="12" max="12" width="19.5" customWidth="1"/>
     <col min="13" max="13" width="25.6640625" customWidth="1"/>
@@ -661,6 +663,9 @@
       <c r="G2">
         <v>30.08</v>
       </c>
+      <c r="H2" s="4">
+        <v>20000</v>
+      </c>
       <c r="I2">
         <v>0.52</v>
       </c>
@@ -702,6 +707,9 @@
       <c r="G3">
         <v>30.08</v>
       </c>
+      <c r="H3" s="4">
+        <v>20000</v>
+      </c>
       <c r="I3">
         <v>0.52</v>
       </c>
@@ -743,6 +751,10 @@
       <c r="G4">
         <v>29.425000000000001</v>
       </c>
+      <c r="H4">
+        <f>AVERAGE(20000, 20000, 12300, 15010)</f>
+        <v>16827.5</v>
+      </c>
       <c r="I4">
         <v>0.65</v>
       </c>
@@ -781,6 +793,9 @@
       <c r="G5">
         <v>29.475000000000001</v>
       </c>
+      <c r="H5" s="4">
+        <v>20000</v>
+      </c>
       <c r="I5">
         <v>0.55000000000000004</v>
       </c>
@@ -822,6 +837,9 @@
       <c r="G6">
         <v>29.475000000000001</v>
       </c>
+      <c r="H6" s="4">
+        <v>20000</v>
+      </c>
       <c r="I6">
         <v>0.55000000000000004</v>
       </c>
@@ -860,6 +878,9 @@
       <c r="G7">
         <v>31.875</v>
       </c>
+      <c r="H7" s="4">
+        <v>20000</v>
+      </c>
       <c r="I7">
         <v>0.9</v>
       </c>
@@ -898,6 +919,10 @@
       <c r="G8">
         <v>23.95</v>
       </c>
+      <c r="H8">
+        <f>AVERAGE(20000, 12250, 20000, 20000)</f>
+        <v>18062.5</v>
+      </c>
       <c r="I8">
         <v>1.0499999999999998</v>
       </c>
@@ -936,6 +961,10 @@
       <c r="G9">
         <v>23.95</v>
       </c>
+      <c r="H9">
+        <f t="shared" ref="H9:H11" si="0">AVERAGE(20000, 12250, 20000, 20000)</f>
+        <v>18062.5</v>
+      </c>
       <c r="I9">
         <v>1.0499999999999998</v>
       </c>
@@ -974,6 +1003,10 @@
       <c r="G10">
         <v>23.95</v>
       </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>18062.5</v>
+      </c>
       <c r="I10">
         <v>1.0499999999999998</v>
       </c>
@@ -1012,6 +1045,10 @@
       <c r="G11">
         <v>23.95</v>
       </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>18062.5</v>
+      </c>
       <c r="I11">
         <v>1.0499999999999998</v>
       </c>
@@ -1050,6 +1087,9 @@
       <c r="G12">
         <v>27.274999999999999</v>
       </c>
+      <c r="H12" s="4">
+        <v>20000</v>
+      </c>
       <c r="I12">
         <v>1.5750000000000002</v>
       </c>
@@ -1088,6 +1128,10 @@
       <c r="G13">
         <v>22.074999999999999</v>
       </c>
+      <c r="H13">
+        <f>AVERAGE(14180, 18260, 13890, 10880)</f>
+        <v>14302.5</v>
+      </c>
       <c r="I13">
         <v>0.05</v>
       </c>
@@ -1126,6 +1170,10 @@
       <c r="G14">
         <v>17.149999999999999</v>
       </c>
+      <c r="H14">
+        <f>AVERAGE(11170, 8601, 5480, 5930)</f>
+        <v>7795.25</v>
+      </c>
       <c r="I14">
         <v>0</v>
       </c>
@@ -1164,6 +1212,9 @@
       <c r="G15">
         <v>24.25</v>
       </c>
+      <c r="H15" s="4">
+        <v>20000</v>
+      </c>
       <c r="I15">
         <v>1.4</v>
       </c>
@@ -1201,6 +1252,10 @@
       </c>
       <c r="G16">
         <v>17.774999999999999</v>
+      </c>
+      <c r="H16">
+        <f>AVERAGE(13830, 14900, 8290, 3790)</f>
+        <v>10202.5</v>
       </c>
       <c r="I16">
         <v>0.82499999999999996</v>
@@ -1240,6 +1295,9 @@
       <c r="G17">
         <v>20.85</v>
       </c>
+      <c r="H17" s="4">
+        <v>20000</v>
+      </c>
       <c r="I17">
         <v>1</v>
       </c>
@@ -1278,6 +1336,9 @@
       <c r="G18">
         <v>24.924999999999997</v>
       </c>
+      <c r="H18" s="4">
+        <v>20000</v>
+      </c>
       <c r="I18">
         <v>1.45</v>
       </c>
@@ -1316,6 +1377,10 @@
       <c r="G19">
         <v>18.274999999999999</v>
       </c>
+      <c r="H19">
+        <f>AVERAGE(4790, 3030, 8860, 11530)</f>
+        <v>7052.5</v>
+      </c>
       <c r="I19">
         <v>0.90000000000000013</v>
       </c>
@@ -1354,6 +1419,10 @@
       <c r="G20">
         <v>18.274999999999999</v>
       </c>
+      <c r="H20">
+        <f>AVERAGE(4790, 3030, 8860, 11530)</f>
+        <v>7052.5</v>
+      </c>
       <c r="I20">
         <v>0.90000000000000013</v>
       </c>
@@ -1392,6 +1461,10 @@
       <c r="G21">
         <v>18.125</v>
       </c>
+      <c r="H21">
+        <f>AVERAGE(11530, 14420, 13820, 12770)</f>
+        <v>13135</v>
+      </c>
       <c r="I21">
         <v>1.3250000000000002</v>
       </c>
@@ -1430,6 +1503,10 @@
       <c r="G22">
         <v>21.674999999999997</v>
       </c>
+      <c r="H22">
+        <f>AVERAGE(20000,20000,16960, 10780)</f>
+        <v>16935</v>
+      </c>
       <c r="I22">
         <v>0.67500000000000004</v>
       </c>
@@ -1468,6 +1545,10 @@
       <c r="G23">
         <v>19.649999999999999</v>
       </c>
+      <c r="H23">
+        <f>AVERAGE(5690, 6801, 13890, 10140)</f>
+        <v>9130.25</v>
+      </c>
       <c r="I23">
         <v>0.5</v>
       </c>
@@ -1506,6 +1587,9 @@
       <c r="G24">
         <v>27.25</v>
       </c>
+      <c r="H24">
+        <v>20000</v>
+      </c>
       <c r="I24">
         <v>0.3</v>
       </c>
@@ -1544,6 +1628,9 @@
       <c r="G25">
         <v>31.6</v>
       </c>
+      <c r="H25">
+        <v>20000</v>
+      </c>
       <c r="I25">
         <v>1.45</v>
       </c>
@@ -1585,6 +1672,9 @@
       <c r="G26">
         <v>24.7</v>
       </c>
+      <c r="H26">
+        <v>20000</v>
+      </c>
       <c r="I26">
         <v>2.7250000000000005</v>
       </c>
@@ -1623,6 +1713,9 @@
       <c r="G27">
         <v>21.4</v>
       </c>
+      <c r="H27">
+        <v>20000</v>
+      </c>
       <c r="I27">
         <v>2.25</v>
       </c>
@@ -1661,6 +1754,10 @@
       <c r="G28">
         <v>20.375</v>
       </c>
+      <c r="H28">
+        <f>AVERAGE(14070, 16070, 20000, 20000)</f>
+        <v>17535</v>
+      </c>
       <c r="I28">
         <v>2.15</v>
       </c>
@@ -1699,6 +1796,9 @@
       <c r="G29">
         <v>25.725000000000001</v>
       </c>
+      <c r="H29" s="4">
+        <v>20000</v>
+      </c>
       <c r="I29">
         <v>2.5</v>
       </c>
@@ -1737,6 +1837,9 @@
       <c r="G30">
         <v>23.875</v>
       </c>
+      <c r="H30" s="4">
+        <v>20000</v>
+      </c>
       <c r="I30">
         <v>2.6</v>
       </c>
@@ -1775,6 +1878,9 @@
       <c r="G31">
         <v>23.875</v>
       </c>
+      <c r="H31" s="4">
+        <v>20000</v>
+      </c>
       <c r="I31">
         <v>2.6</v>
       </c>
@@ -1816,6 +1922,9 @@
       <c r="G32">
         <v>22.175000000000001</v>
       </c>
+      <c r="H32" s="4">
+        <v>20000</v>
+      </c>
       <c r="I32">
         <v>2.5750000000000002</v>
       </c>
@@ -1854,6 +1963,10 @@
       <c r="G33">
         <v>19.700000000000003</v>
       </c>
+      <c r="H33">
+        <f>AVERAGE(9110, 15510, 18380, 20000)</f>
+        <v>15750</v>
+      </c>
       <c r="I33">
         <v>0.77500000000000002</v>
       </c>
@@ -1895,6 +2008,10 @@
       <c r="G34">
         <v>19.700000000000003</v>
       </c>
+      <c r="H34">
+        <f t="shared" ref="H34:H35" si="1">AVERAGE(9110, 15510, 18380, 20000)</f>
+        <v>15750</v>
+      </c>
       <c r="I34">
         <v>0.77500000000000002</v>
       </c>
@@ -1933,6 +2050,10 @@
       <c r="G35">
         <v>19.700000000000003</v>
       </c>
+      <c r="H35">
+        <f t="shared" si="1"/>
+        <v>15750</v>
+      </c>
       <c r="I35">
         <v>0.77500000000000002</v>
       </c>
@@ -1974,6 +2095,9 @@
       <c r="G36">
         <v>25.95</v>
       </c>
+      <c r="H36" s="4">
+        <v>20000</v>
+      </c>
       <c r="I36">
         <v>1.375</v>
       </c>
@@ -2015,6 +2139,9 @@
       <c r="G37">
         <v>25.375</v>
       </c>
+      <c r="H37" s="4">
+        <v>20000</v>
+      </c>
       <c r="I37">
         <v>2.2999999999999998</v>
       </c>
@@ -2055,6 +2182,9 @@
       </c>
       <c r="G38">
         <v>22.299999999999997</v>
+      </c>
+      <c r="H38" s="4">
+        <v>20000</v>
       </c>
       <c r="I38">
         <v>2.1749999999999998</v>
@@ -2079,7 +2209,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1284E74-CE0A-214D-889F-E511955B9768}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:U38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -2090,9 +2220,10 @@
     <col min="14" max="14" width="19.33203125" customWidth="1"/>
     <col min="15" max="15" width="23.1640625" customWidth="1"/>
     <col min="16" max="16" width="24.6640625" customWidth="1"/>
+    <col min="21" max="21" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -2142,7 +2273,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2164,6 +2295,9 @@
       <c r="G2">
         <v>30.08</v>
       </c>
+      <c r="H2" s="4">
+        <v>20000</v>
+      </c>
       <c r="I2">
         <v>0.52</v>
       </c>
@@ -2188,8 +2322,9 @@
       <c r="P2">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U2" s="4"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>3</v>
       </c>
@@ -2211,6 +2346,10 @@
       <c r="G3">
         <v>29.425000000000001</v>
       </c>
+      <c r="H3">
+        <f>AVERAGE(20000, 20000, 12300, 15010)</f>
+        <v>16827.5</v>
+      </c>
       <c r="I3">
         <v>0.65</v>
       </c>
@@ -2235,8 +2374,9 @@
       <c r="P3">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U3" s="4"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>4</v>
       </c>
@@ -2258,6 +2398,9 @@
       <c r="G4">
         <v>29.475000000000001</v>
       </c>
+      <c r="H4" s="4">
+        <v>20000</v>
+      </c>
       <c r="I4">
         <v>0.55000000000000004</v>
       </c>
@@ -2283,7 +2426,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>6</v>
       </c>
@@ -2305,6 +2448,9 @@
       <c r="G5">
         <v>31.875</v>
       </c>
+      <c r="H5" s="4">
+        <v>20000</v>
+      </c>
       <c r="I5">
         <v>0.9</v>
       </c>
@@ -2329,8 +2475,9 @@
       <c r="P5">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U5" s="4"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>7</v>
       </c>
@@ -2352,6 +2499,10 @@
       <c r="G6">
         <v>23.95</v>
       </c>
+      <c r="H6">
+        <f>AVERAGE(20000, 12250, 20000, 20000)</f>
+        <v>18062.5</v>
+      </c>
       <c r="I6">
         <v>1.0499999999999998</v>
       </c>
@@ -2376,8 +2527,9 @@
       <c r="P6">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U6" s="4"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>11</v>
       </c>
@@ -2399,6 +2551,9 @@
       <c r="G7">
         <v>27.274999999999999</v>
       </c>
+      <c r="H7" s="4">
+        <v>20000</v>
+      </c>
       <c r="I7">
         <v>1.5750000000000002</v>
       </c>
@@ -2423,8 +2578,9 @@
       <c r="P7">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U7" s="4"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>12</v>
       </c>
@@ -2446,6 +2602,10 @@
       <c r="G8">
         <v>22.074999999999999</v>
       </c>
+      <c r="H8">
+        <f>AVERAGE(14180, 18260, 13890, 10880)</f>
+        <v>14302.5</v>
+      </c>
       <c r="I8">
         <v>0.05</v>
       </c>
@@ -2471,7 +2631,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>13</v>
       </c>
@@ -2493,6 +2653,10 @@
       <c r="G9">
         <v>17.149999999999999</v>
       </c>
+      <c r="H9">
+        <f>AVERAGE(11170, 8601, 5480, 5930)</f>
+        <v>7795.25</v>
+      </c>
       <c r="I9">
         <v>0</v>
       </c>
@@ -2518,7 +2682,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>14</v>
       </c>
@@ -2540,6 +2704,9 @@
       <c r="G10">
         <v>24.25</v>
       </c>
+      <c r="H10" s="4">
+        <v>20000</v>
+      </c>
       <c r="I10">
         <v>1.4</v>
       </c>
@@ -2565,7 +2732,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>15</v>
       </c>
@@ -2587,6 +2754,10 @@
       <c r="G11">
         <v>17.774999999999999</v>
       </c>
+      <c r="H11">
+        <f>AVERAGE(13830, 14900, 8290, 3790)</f>
+        <v>10202.5</v>
+      </c>
       <c r="I11">
         <v>0.82499999999999996</v>
       </c>
@@ -2612,7 +2783,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>16</v>
       </c>
@@ -2634,6 +2805,9 @@
       <c r="G12">
         <v>20.85</v>
       </c>
+      <c r="H12" s="4">
+        <v>20000</v>
+      </c>
       <c r="I12">
         <v>1</v>
       </c>
@@ -2658,8 +2832,9 @@
       <c r="P12">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U12" s="4"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>17</v>
       </c>
@@ -2681,6 +2856,9 @@
       <c r="G13">
         <v>24.924999999999997</v>
       </c>
+      <c r="H13" s="4">
+        <v>20000</v>
+      </c>
       <c r="I13">
         <v>1.45</v>
       </c>
@@ -2706,7 +2884,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>18</v>
       </c>
@@ -2728,6 +2906,10 @@
       <c r="G14">
         <v>18.274999999999999</v>
       </c>
+      <c r="H14">
+        <f>AVERAGE(4790, 3030, 8860, 11530)</f>
+        <v>7052.5</v>
+      </c>
       <c r="I14">
         <v>0.90000000000000013</v>
       </c>
@@ -2753,7 +2935,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>20</v>
       </c>
@@ -2775,6 +2957,10 @@
       <c r="G15">
         <v>18.125</v>
       </c>
+      <c r="H15">
+        <f>AVERAGE(11530, 14420, 13820, 12770)</f>
+        <v>13135</v>
+      </c>
       <c r="I15">
         <v>1.3250000000000002</v>
       </c>
@@ -2799,8 +2985,9 @@
       <c r="P15">
         <v>7</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U15" s="4"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>21</v>
       </c>
@@ -2822,6 +3009,10 @@
       <c r="G16">
         <v>21.674999999999997</v>
       </c>
+      <c r="H16">
+        <f>AVERAGE(20000,20000,16960, 10780)</f>
+        <v>16935</v>
+      </c>
       <c r="I16">
         <v>0.67500000000000004</v>
       </c>
@@ -2847,7 +3038,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>22</v>
       </c>
@@ -2869,6 +3060,10 @@
       <c r="G17">
         <v>19.649999999999999</v>
       </c>
+      <c r="H17">
+        <f>AVERAGE(5690, 6801, 13890, 10140)</f>
+        <v>9130.25</v>
+      </c>
       <c r="I17">
         <v>0.5</v>
       </c>
@@ -2893,8 +3088,9 @@
       <c r="P17">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U17" s="4"/>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>23</v>
       </c>
@@ -2916,6 +3112,9 @@
       <c r="G18">
         <v>27.25</v>
       </c>
+      <c r="H18">
+        <v>20000</v>
+      </c>
       <c r="I18">
         <v>0.3</v>
       </c>
@@ -2940,8 +3139,9 @@
       <c r="P18">
         <v>5</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="U18" s="4"/>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>24</v>
       </c>
@@ -2963,6 +3163,9 @@
       <c r="G19">
         <v>31.6</v>
       </c>
+      <c r="H19">
+        <v>20000</v>
+      </c>
       <c r="I19">
         <v>1.45</v>
       </c>
@@ -2988,7 +3191,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>25</v>
       </c>
@@ -3010,6 +3213,9 @@
       <c r="G20">
         <v>24.7</v>
       </c>
+      <c r="H20">
+        <v>20000</v>
+      </c>
       <c r="I20">
         <v>2.7250000000000005</v>
       </c>
@@ -3035,7 +3241,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>26</v>
       </c>
@@ -3057,6 +3263,9 @@
       <c r="G21">
         <v>21.4</v>
       </c>
+      <c r="H21">
+        <v>20000</v>
+      </c>
       <c r="I21">
         <v>2.25</v>
       </c>
@@ -3082,7 +3291,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>27</v>
       </c>
@@ -3104,6 +3313,10 @@
       <c r="G22">
         <v>20.375</v>
       </c>
+      <c r="H22">
+        <f>AVERAGE(14070, 16070, 20000, 20000)</f>
+        <v>17535</v>
+      </c>
       <c r="I22">
         <v>2.15</v>
       </c>
@@ -3129,7 +3342,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>28</v>
       </c>
@@ -3151,6 +3364,9 @@
       <c r="G23">
         <v>25.725000000000001</v>
       </c>
+      <c r="H23" s="4">
+        <v>20000</v>
+      </c>
       <c r="I23">
         <v>2.5</v>
       </c>
@@ -3176,7 +3392,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>29</v>
       </c>
@@ -3198,6 +3414,9 @@
       <c r="G24">
         <v>23.875</v>
       </c>
+      <c r="H24" s="4">
+        <v>20000</v>
+      </c>
       <c r="I24">
         <v>2.6</v>
       </c>
@@ -3223,7 +3442,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>31</v>
       </c>
@@ -3245,6 +3464,9 @@
       <c r="G25">
         <v>22.175000000000001</v>
       </c>
+      <c r="H25" s="4">
+        <v>20000</v>
+      </c>
       <c r="I25">
         <v>2.5750000000000002</v>
       </c>
@@ -3270,7 +3492,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>32</v>
       </c>
@@ -3292,6 +3514,10 @@
       <c r="G26">
         <v>19.700000000000003</v>
       </c>
+      <c r="H26">
+        <f>AVERAGE(9110, 15510, 18380, 20000)</f>
+        <v>15750</v>
+      </c>
       <c r="I26">
         <v>0.77500000000000002</v>
       </c>
@@ -3317,7 +3543,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>35</v>
       </c>
@@ -3339,6 +3565,9 @@
       <c r="G27">
         <v>25.95</v>
       </c>
+      <c r="H27" s="4">
+        <v>20000</v>
+      </c>
       <c r="I27">
         <v>1.375</v>
       </c>
@@ -3364,7 +3593,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>36</v>
       </c>
@@ -3386,6 +3615,9 @@
       <c r="G28">
         <v>25.375</v>
       </c>
+      <c r="H28" s="4">
+        <v>20000</v>
+      </c>
       <c r="I28">
         <v>2.2999999999999998</v>
       </c>
@@ -3411,7 +3643,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>37</v>
       </c>
@@ -3433,6 +3665,9 @@
       <c r="G29">
         <v>22.299999999999997</v>
       </c>
+      <c r="H29" s="4">
+        <v>20000</v>
+      </c>
       <c r="I29">
         <v>2.1749999999999998</v>
       </c>
@@ -3457,6 +3692,25 @@
       <c r="P29">
         <v>8</v>
       </c>
+      <c r="U29" s="4"/>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="U30" s="4"/>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="U31" s="4"/>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="U32" s="4"/>
+    </row>
+    <row r="36" spans="21:21" x14ac:dyDescent="0.2">
+      <c r="U36" s="4"/>
+    </row>
+    <row r="37" spans="21:21" x14ac:dyDescent="0.2">
+      <c r="U37" s="4"/>
+    </row>
+    <row r="38" spans="21:21" x14ac:dyDescent="0.2">
+      <c r="U38" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
rename scripts, and sort diversity index
</commit_message>
<xml_diff>
--- a/spreadsheets/P_lanceolata.xlsx
+++ b/spreadsheets/P_lanceolata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sallyborrowman/R_projects/temporal_pollinators/spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EE88B7-4708-4943-946F-9FC35F34C279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67843B3-AF6C-DD45-892F-DE15D1B185B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="17400" activeTab="1" xr2:uid="{DD5157BD-592B-EF4A-95FF-FB179A475922}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{DD5157BD-592B-EF4A-95FF-FB179A475922}"/>
   </bookViews>
   <sheets>
     <sheet name="pollinator_data_raw" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="54">
   <si>
     <t>Temp_shade</t>
   </si>
@@ -3733,6 +3733,7 @@
     <col min="9" max="9" width="24.83203125" customWidth="1"/>
     <col min="10" max="10" width="27.1640625" customWidth="1"/>
     <col min="11" max="11" width="30.6640625" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -3795,14 +3796,14 @@
       <c r="H2">
         <v>22</v>
       </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>15</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -3812,8 +3813,8 @@
       <c r="B3">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
-        <v>15</v>
+      <c r="C3">
+        <v>0</v>
       </c>
       <c r="D3">
         <v>78</v>
@@ -3833,11 +3834,11 @@
       <c r="I3">
         <v>2</v>
       </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>15</v>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -3847,8 +3848,8 @@
       <c r="B4">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
-        <v>15</v>
+      <c r="C4">
+        <v>0</v>
       </c>
       <c r="D4">
         <v>71</v>
@@ -3865,14 +3866,14 @@
       <c r="H4">
         <v>4</v>
       </c>
-      <c r="I4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" t="s">
-        <v>15</v>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -3882,8 +3883,8 @@
       <c r="B5">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
-        <v>15</v>
+      <c r="C5">
+        <v>0</v>
       </c>
       <c r="D5">
         <v>37</v>
@@ -3900,14 +3901,14 @@
       <c r="H5">
         <v>5</v>
       </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" t="s">
-        <v>15</v>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -3917,8 +3918,8 @@
       <c r="B6">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
-        <v>15</v>
+      <c r="C6">
+        <v>0</v>
       </c>
       <c r="D6">
         <v>67</v>
@@ -3935,14 +3936,14 @@
       <c r="H6">
         <v>4</v>
       </c>
-      <c r="I6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K6" t="s">
-        <v>15</v>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -3952,8 +3953,8 @@
       <c r="B7">
         <v>23</v>
       </c>
-      <c r="C7" t="s">
-        <v>15</v>
+      <c r="C7">
+        <v>0</v>
       </c>
       <c r="D7">
         <v>86</v>
@@ -3970,14 +3971,14 @@
       <c r="H7">
         <v>3</v>
       </c>
-      <c r="I7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7" t="s">
-        <v>15</v>
-      </c>
-      <c r="K7" t="s">
-        <v>15</v>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -3987,8 +3988,8 @@
       <c r="B8">
         <v>26</v>
       </c>
-      <c r="C8" t="s">
-        <v>15</v>
+      <c r="C8">
+        <v>0</v>
       </c>
       <c r="D8">
         <v>73</v>
@@ -3996,8 +3997,8 @@
       <c r="E8">
         <v>204</v>
       </c>
-      <c r="F8" t="s">
-        <v>15</v>
+      <c r="F8">
+        <v>0</v>
       </c>
       <c r="G8">
         <v>60</v>
@@ -4005,14 +4006,14 @@
       <c r="H8">
         <v>7</v>
       </c>
-      <c r="I8" t="s">
-        <v>15</v>
-      </c>
-      <c r="J8" t="s">
-        <v>15</v>
-      </c>
-      <c r="K8" t="s">
-        <v>15</v>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -4022,8 +4023,8 @@
       <c r="B9">
         <v>17</v>
       </c>
-      <c r="C9" t="s">
-        <v>15</v>
+      <c r="C9">
+        <v>0</v>
       </c>
       <c r="D9">
         <v>41</v>
@@ -4031,8 +4032,8 @@
       <c r="E9">
         <v>180</v>
       </c>
-      <c r="F9" t="s">
-        <v>15</v>
+      <c r="F9">
+        <v>0</v>
       </c>
       <c r="G9">
         <v>72</v>
@@ -4040,14 +4041,14 @@
       <c r="H9">
         <v>6</v>
       </c>
-      <c r="I9" t="s">
-        <v>15</v>
-      </c>
-      <c r="J9" t="s">
-        <v>15</v>
-      </c>
-      <c r="K9" t="s">
-        <v>15</v>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
@@ -4057,8 +4058,8 @@
       <c r="B10">
         <v>14</v>
       </c>
-      <c r="C10" t="s">
-        <v>15</v>
+      <c r="C10">
+        <v>0</v>
       </c>
       <c r="D10">
         <v>38</v>
@@ -4066,8 +4067,8 @@
       <c r="E10">
         <v>54</v>
       </c>
-      <c r="F10" t="s">
-        <v>15</v>
+      <c r="F10">
+        <v>0</v>
       </c>
       <c r="G10">
         <v>32</v>
@@ -4075,14 +4076,14 @@
       <c r="H10">
         <v>5</v>
       </c>
-      <c r="I10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J10" t="s">
-        <v>15</v>
-      </c>
-      <c r="K10" t="s">
-        <v>15</v>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
@@ -4092,17 +4093,17 @@
       <c r="B11">
         <v>18</v>
       </c>
-      <c r="C11" t="s">
-        <v>15</v>
+      <c r="C11">
+        <v>0</v>
       </c>
       <c r="D11">
         <v>21</v>
       </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" t="s">
-        <v>15</v>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
       </c>
       <c r="G11">
         <v>61</v>
@@ -4110,84 +4111,84 @@
       <c r="H11">
         <v>5</v>
       </c>
-      <c r="I11" t="s">
-        <v>15</v>
-      </c>
-      <c r="J11" t="s">
-        <v>15</v>
-      </c>
-      <c r="K11" t="s">
-        <v>15</v>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>46216</v>
       </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" t="s">
-        <v>15</v>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
       </c>
       <c r="F12">
         <v>57</v>
       </c>
-      <c r="G12" t="s">
-        <v>15</v>
+      <c r="G12">
+        <v>0</v>
       </c>
       <c r="H12">
         <v>7</v>
       </c>
-      <c r="I12" t="s">
-        <v>15</v>
-      </c>
-      <c r="J12" t="s">
-        <v>15</v>
-      </c>
-      <c r="K12" t="s">
-        <v>15</v>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>46217</v>
       </c>
-      <c r="B13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" t="s">
-        <v>15</v>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
       </c>
       <c r="F13">
         <v>56</v>
       </c>
-      <c r="G13" t="s">
-        <v>15</v>
+      <c r="G13">
+        <v>0</v>
       </c>
       <c r="H13">
         <v>6</v>
       </c>
-      <c r="I13" t="s">
-        <v>15</v>
-      </c>
-      <c r="J13" t="s">
-        <v>15</v>
-      </c>
-      <c r="K13" t="s">
-        <v>15</v>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
@@ -4197,14 +4198,14 @@
       <c r="B14">
         <v>2</v>
       </c>
-      <c r="C14" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" t="s">
-        <v>15</v>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
       </c>
       <c r="F14">
         <v>25</v>
@@ -4215,14 +4216,14 @@
       <c r="H14">
         <v>7</v>
       </c>
-      <c r="I14" t="s">
-        <v>15</v>
+      <c r="I14">
+        <v>0</v>
       </c>
       <c r="J14">
         <v>699</v>
       </c>
-      <c r="K14" t="s">
-        <v>15</v>
+      <c r="K14">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
@@ -4232,26 +4233,26 @@
       <c r="B15">
         <v>2</v>
       </c>
-      <c r="C15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" t="s">
-        <v>15</v>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
       </c>
       <c r="F15">
         <v>23</v>
       </c>
-      <c r="G15" t="s">
-        <v>15</v>
+      <c r="G15">
+        <v>0</v>
       </c>
       <c r="H15">
         <v>8</v>
       </c>
-      <c r="I15" t="s">
-        <v>15</v>
+      <c r="I15">
+        <v>0</v>
       </c>
       <c r="J15">
         <v>399</v>

</xml_diff>